<commit_message>
feat: add magalu_bot interface
</commit_message>
<xml_diff>
--- a/aflmain/links_afiliados_magalu.xlsx
+++ b/aflmain/links_afiliados_magalu.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -488,29 +488,19 @@
           <t>https://www.magazinevoce.com.br/magazineblackriseco/armario-de-cozinha-compacta-aramoveis-cleo-8-portas/p/235418000/mo/mcoz/</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>R$ 680,00</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>ou R$ 522,49</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>REVISAR</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:15:33</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Não foi possível obter o link de afiliado.</t>
         </is>
       </c>
     </row>
@@ -533,31 +523,6 @@
           <t>https://magazineluiza.onelink.me/589508454/nk0eeuch</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>R$ 889,99</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>ou R$ 710,99</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:15:49</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Link de afiliado obtido com sucesso.</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -578,31 +543,6 @@
           <t>https://magazineluiza.onelink.me/589508454/53vlf84b</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>R$ 615,88</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>ou R$ 431,11</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:15:58</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Link de afiliado obtido com sucesso.</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -623,31 +563,6 @@
           <t>https://magazineluiza.onelink.me/589508454/delyqvg9</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>R$ 919,99</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>ou R$ 737,99</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:16:09</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Link de afiliado obtido com sucesso.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -663,29 +578,19 @@
           <t>https://www.magazinevoce.com.br/magazineblackriseco/armario-de-cozinha-aereo-itatiaia-rose-arm-105-3-portas-105x40cm/p/237989400/mo/moac/</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>R$ 300,00</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>ou R$ 256,49</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>REVISAR</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:16:33</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Não foi possível obter o link de afiliado.</t>
         </is>
       </c>
     </row>
@@ -708,31 +613,6 @@
           <t>https://magazineluiza.onelink.me/589508454/e1k0pbkp</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>R$ 799,99</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>ou R$ 611,99</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:16:44</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Link de afiliado obtido com sucesso.</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -748,29 +628,19 @@
           <t>https://www.magazinevoce.com.br/magazineblackriseco/armario-de-cozinha-compacta-demobile-select-com-balcao-nicho-para-micro-ondas-6-portas-2-gavetas/p/234470600/mo/moac/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>R$ 1.099,00</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>ou R$ 759,99</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>REVISAR</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:17:10</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Não foi possível obter o link de afiliado.</t>
         </is>
       </c>
     </row>
@@ -788,31 +658,6 @@
           <t>https://www.magazinevoce.com.br/magazineblackriseco/armario-de-cozinha-compacta-itatiaia-amanda-aco-com-balcao-10-portas-1-gaveta/p/237989500/mo/moac/</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>R$ 1.199,00</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>ou R$ 989,99</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:17:33</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Não foi possível obter o link de afiliado.</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -833,26 +678,6 @@
           <t>https://magazineluiza.onelink.me/589508454/ktwblbe0</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>ou R$ 494,99</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:17:51</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Link de afiliado obtido com sucesso.</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -873,31 +698,6 @@
           <t>https://magazineluiza.onelink.me/589508454/c2ocbzve</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>R$ 539,99</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>ou R$ 443,69</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:18:04</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Link de afiliado obtido com sucesso.</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -918,31 +718,6 @@
           <t>https://magazineluiza.onelink.me/589508454/xddw0uy8</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>R$ 739,99</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>ou R$ 611,99</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:18:17</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Link de afiliado obtido com sucesso.</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -963,22 +738,847 @@
           <t>https://magazineluiza.onelink.me/589508454/ey1ubse9</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>ou R$ 594,99</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>21/08/2026 09:18:36</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/jogo-marvels-spider-man-2-playstation-5/p/237987800/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>R$ 299,90</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>ou R$ 188,95</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:43:44</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Não foi possível obter o link de afiliado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/jogo-the-last-of-us-2-remastered-ps5-midia-fisica-portugues-playstation/p/ce09340880/ga/jaco/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/qneyhr8v</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ou R$ 353,31</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:44:04</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/red-dead-redemption-2-ps4-midia-fisica-playstation/p/ad1ahb77jj/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/n5b734fm</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ou R$ 149,57</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:44:21</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/jogo-a-ascensao-do-ronin-standard-edition-playstation-5-midia-fisica-sony/p/kff933d4d0/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/xty5v84b</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>R$ 299,90</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ou R$ 199,90</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:44:34</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/dark-souls-trilogy-ps4-eur-midia-fisica-playstation/p/cj01h4b5f5/ga/drks/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/ewhxp8dt</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>ou R$ 255,17</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:44:48</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/call-of-duty-black-ops-7-ps5-midia-fisica-playstation/p/hgjjhdd2fh/ga/otga/</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/39bdkhei</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ou R$ 299,17</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:45:02</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/just-dance-2020-para-ps4-ubisoft/p/043184800/ga/juda/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>R$ 179,90</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ou R$ 138,70</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>REVISAR</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:45:28</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Não foi possível obter o link de afiliado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/cuphead-ps4-midia-fisica-playstation/p/cj978d3ggk/ga/javt/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/p8eprtwv</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>ou R$ 167,17</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:45:47</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>9</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/warhammer-40000-space-marine-2-ps5-midia-fisica-playstation/p/jekd3b6k8k/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/r2tgyxd1</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>ou R$ 219,97</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:46:04</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/jogo-de-video-atari-stuntman-playstation-2-novo/p/fg3212d6h6/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/wgb0yqne</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>R$ 329,17</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>ou R$ 310,34</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:46:14</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>11</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/videogame-cuphead-playstation-4-com-cooperacao-local-para-2-jogadores-iam8bit/p/khbfkdg8h9/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/7ffkmllk</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>R$ 343,74</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>ou R$ 320,86</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:46:23</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>12</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/jogo-eletronico-jurassic-world-evolution-2-playstation-5-sold-out/p/dfebch02e3/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/d9lx7ab7</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>R$ 380,46</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>ou R$ 357,68</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:46:36</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>13</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/jogo-eletronico-sniper-ghost-warrior-contracts-2-playstation-5-ci-games/p/cj7b8bdj58/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/jrrco1wt</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>R$ 312,18</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>ou R$ 268,26</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:46:51</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>14</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/jogo-de-video-lego-marvel-superheroes-2-playstation-4-wb-games/p/hc56bd1186/ga/lego/</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/f2k5xcdp</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>R$ 260,37</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>ou R$ 241,96</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:47:00</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>15</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/videogame-capcom-resident-evil-2-para-playstation-5/p/jh5f76kc85/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/xydrpaj6</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>R$ 234,91</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>ou R$ 215,66</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:47:11</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>16</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/invincible-vs-ps5-midia-fisica-playstation/p/cbe84efc59/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/fqpnwh5s</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>ou R$ 263,97</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:47:28</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>17</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/destroy-all-humans-2-reprobed-ps5-eur-midia-fisica-playstation/p/ja5k6k1e79/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/r1u2lhik</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>R$ 114,37</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:47:45</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>18</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/jogo-eletronico-marvel-s-spider-man-2-playstation/p/ja6626h7c9/ga/jaco/</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/l5t4c571</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>R$ 563,03</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>ou R$ 536,52</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:47:59</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>19</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/jogo-de-video-atari-backyard-basketball-playstation-2/p/heckjc2486/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/wijvfa2t</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>R$ 271,63</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>ou R$ 247,22</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:48:07</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Link de afiliado obtido com sucesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>jogos playstation 2</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>20</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.magazinevoce.com.br/magazineblackriseco/fatal-fury-city-of-the-wolves-special-edition-ps4-midia-fisica-playstation/p/bebk01hgf2/ga/jgpn/</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://magazineluiza.onelink.me/589508454/u4mdrexd</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>ou R$ 184,77</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>21/08/2026 11:48:21</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
         <is>
           <t>Link de afiliado obtido com sucesso.</t>
         </is>

</xml_diff>